<commit_message>
Update relative lung volume to be referenced to FRC. Update mechanical ventilation SDK example for a sensor control system.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/CSTARS/CSTARS.xlsx
+++ b/data/human/adult/validation/Scenarios/CSTARS/CSTARS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\CSTARS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99B92EAC-9656-497E-85E5-4ACF6BCC0140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649538A5-929B-47F0-954D-1BB634B0E5FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27780" yWindow="5415" windowWidth="28455" windowHeight="24405" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29205" yWindow="4410" windowWidth="28230" windowHeight="25455" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="Scenario6" sheetId="6" r:id="rId6"/>
     <sheet name="Scenario7" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -739,57 +739,6 @@
 }</t>
   </si>
   <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 40, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.9, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 15, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 18, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 600, "Unit": "mL" } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>Change in ventilator settings.
-Learning Objectives:
- - Recognize and address fall in oxygenation
- - Recognize and if required - address increase in PIP to maintain lung protection. (Pplat &lt; 30 cm H2O) (reduce VT)
- - Increase PEEP (first choice) and/or FIO2
-Recommended Actions:
- - Decrease FiO2 until SpO2 acceptable
- - Then match PEEP to FiO2
- - Decrease tidal volume to get Pplat &lt; 30
-Ventilator settings are updated to:
- - PEEP: 8 -&gt; 14 cmH2O
-| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.6    | NA          | 40           | NA  | 0.9    | 18      | 15            | 0.40 |</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 40, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.9, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 18, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 600, "Unit": "mL" } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>Ventilator settings are:
-&lt;br /&gt;
-| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.6    | NA          | 40           | NA  | 0.9    | 18      | 5            | 0.40 |</t>
-  </si>
-  <si>
     <t>Mild ARDS with Progressive Fall in Oxygenation</t>
   </si>
   <si>
@@ -840,6 +789,57 @@
       { "Compartment": "RightLung", "Severity": { "Scalar0To1": { "Value": 0.6 }}}]
   }}
 }</t>
+  </si>
+  <si>
+    <t>Ventilator settings are:
+&lt;br /&gt;
+| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| VC-CMV | 0.567    | NA          | 27           | NA  | 1.25    | 16      | 5            | 0.4 |</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 27, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.25, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 16, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 567, "Unit": "mL" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 27, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.25, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 15, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 16, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 567, "Unit": "mL" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>Change in ventilator settings.
+Learning Objectives:
+ - Recognize and address fall in oxygenation
+ - Recognize and if required - address increase in PIP to maintain lung protection. (Pplat &lt; 30 cm H2O) (reduce VT)
+ - Increase PEEP (first choice) and/or FIO2
+Recommended Actions:
+ - Decrease FiO2 until SpO2 acceptable
+ - Then match PEEP to FiO2
+ - Decrease tidal volume to get Pplat &lt; 30
+Ventilator settings are updated to:
+ - PEEP: 8 -&gt; 14 cmH2O
+| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| VC-CMV | 0.567    | NA          | 27           | NA  | 1.25    | 16      | 15            | 0.4 |</t>
   </si>
 </sst>
 </file>
@@ -1448,7 +1448,7 @@
     </row>
     <row r="2" spans="1:1024" ht="105.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B2" s="21"/>
       <c r="C2" s="21" t="s">
@@ -1620,7 +1620,7 @@
       <c r="E12" s="25"/>
       <c r="F12" s="25"/>
       <c r="G12" s="9" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -1659,14 +1659,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C15" s="25"/>
       <c r="D15" s="25"/>
       <c r="E15" s="25"/>
       <c r="F15" s="25"/>
       <c r="G15" s="9" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -1675,7 +1675,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C16" s="25"/>
       <c r="D16" s="25"/>
@@ -2044,7 +2044,7 @@
       <c r="E32" s="25"/>
       <c r="F32" s="25"/>
       <c r="G32" s="9" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="H32" s="9"/>
     </row>
@@ -2053,7 +2053,7 @@
         <v>2</v>
       </c>
       <c r="B33" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C33" s="25"/>
       <c r="D33" s="25"/>
@@ -2493,14 +2493,14 @@
         <v>3</v>
       </c>
       <c r="B52" s="25" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C52" s="25"/>
       <c r="D52" s="25"/>
       <c r="E52" s="25"/>
       <c r="F52" s="25"/>
       <c r="G52" s="9" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H52" s="10"/>
     </row>
@@ -2509,7 +2509,7 @@
         <v>3</v>
       </c>
       <c r="B53" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C53" s="25"/>
       <c r="D53" s="25"/>
@@ -3182,7 +3182,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C16" s="25"/>
       <c r="D16" s="25"/>
@@ -3558,7 +3558,7 @@
         <v>2</v>
       </c>
       <c r="B33" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C33" s="25"/>
       <c r="D33" s="25"/>
@@ -3920,7 +3920,7 @@
         <v>3</v>
       </c>
       <c r="B49" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C49" s="25"/>
       <c r="D49" s="25"/>
@@ -4543,7 +4543,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C16" s="25"/>
       <c r="D16" s="25"/>
@@ -9953,7 +9953,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C31" s="25"/>
       <c r="D31" s="25"/>
@@ -24493,7 +24493,7 @@
         <v>3</v>
       </c>
       <c r="B45" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C45" s="25"/>
       <c r="D45" s="25"/>
@@ -31770,12 +31770,12 @@
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B29:F29"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B29:F29"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="E5:F9"/>
@@ -32060,7 +32060,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C16" s="25"/>
       <c r="D16" s="25"/>
@@ -32328,7 +32328,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C28" s="25"/>
       <c r="D28" s="25"/>
@@ -32572,7 +32572,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C39" s="25"/>
       <c r="D39" s="25"/>
@@ -33028,7 +33028,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C16" s="25"/>
       <c r="D16" s="25"/>
@@ -33320,7 +33320,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
@@ -33588,7 +33588,7 @@
         <v>3</v>
       </c>
       <c r="B41" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C41" s="25"/>
       <c r="D41" s="25"/>
@@ -33908,7 +33908,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="25" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C12" s="25"/>
       <c r="D12" s="25"/>
@@ -33956,7 +33956,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C15" s="25"/>
       <c r="D15" s="25"/>
@@ -34296,7 +34296,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C30" s="25"/>
       <c r="D30" s="25"/>
@@ -34564,7 +34564,7 @@
         <v>3</v>
       </c>
       <c r="B42" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C42" s="25"/>
       <c r="D42" s="25"/>
@@ -34915,14 +34915,14 @@
         <v>1</v>
       </c>
       <c r="B14" s="25" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
       <c r="E14" s="25"/>
       <c r="F14" s="25"/>
       <c r="G14" s="9" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="H14" s="10"/>
     </row>
@@ -34931,7 +34931,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C15" s="25"/>
       <c r="D15" s="25"/>
@@ -35287,7 +35287,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C31" s="25"/>
       <c r="D31" s="25"/>
@@ -35555,7 +35555,7 @@
         <v>3</v>
       </c>
       <c r="B43" s="25" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C43" s="25"/>
       <c r="D43" s="25"/>

</xml_diff>

<commit_message>
Rename "apparent" outputs as "clinical" outputs.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/CSTARS/CSTARS.xlsx
+++ b/data/human/adult/validation/Scenarios/CSTARS/CSTARS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\CSTARS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC4A6A2-14D3-46AE-A505-AFAB17A0F159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96BB453-B3BC-40FF-8BCA-FAFBFF6AD250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28170" yWindow="3435" windowWidth="29445" windowHeight="26775" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21705" yWindow="2100" windowWidth="34530" windowHeight="26775" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patients" sheetId="8" r:id="rId1"/>
@@ -1168,34 +1168,16 @@
 &lt;br /&gt;</t>
   </si>
   <si>
-    <t>ApparentShuntFraction</t>
-  </si>
-  <si>
-    <t>ApparentPhysiologicDeadSpaceTidalVolumeRatio</t>
-  </si>
-  <si>
-    <t>VD/VT for mild ARDS (determined from blood gas values)</t>
-  </si>
-  <si>
     <t>QS/QT for mild ARDS (determined from blood gas values)</t>
   </si>
   <si>
-    <t>VD/VT for moderate ARDS (determined from blood gas values)</t>
-  </si>
-  <si>
     <t>QS/QT for moderate ARDS (determined from blood gas values)</t>
   </si>
   <si>
     <t>QS/QT (determined from blood gas values)</t>
   </si>
   <si>
-    <t>VD/VT for moderate COPD (determined from blood gas values)</t>
-  </si>
-  <si>
     <t>QS/QT for moderate COPD (determined from blood gas values)</t>
-  </si>
-  <si>
-    <t>VD/VT for severe ARDS (determined from blood gas values)</t>
   </si>
   <si>
     <t>QS/QT for severe ARDS (determined from blood gas values)</t>
@@ -1439,6 +1421,24 @@
   "InspirationPatientTriggerFlow": { "ScalarVolumePerTime": { "Value": 1.0, "Unit": "L/min"  } }
   }}
 }</t>
+  </si>
+  <si>
+    <t>PhysiologicDeadSpaceTidalVolumeRatio</t>
+  </si>
+  <si>
+    <t>VD/VT for mild ARDS</t>
+  </si>
+  <si>
+    <t>VD/VT for moderate ARDS</t>
+  </si>
+  <si>
+    <t>VD/VT for moderate COPD</t>
+  </si>
+  <si>
+    <t>VD/VT for severe ARDS</t>
+  </si>
+  <si>
+    <t>ClinicalShuntFraction</t>
   </si>
 </sst>
 </file>
@@ -1957,10 +1957,28 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1982,24 +2000,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2811,42 +2811,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
       <c r="AMG1" s="13"/>
       <c r="AMH1" s="13"/>
       <c r="AMI1" s="13"/>
       <c r="AMJ1" s="13"/>
     </row>
     <row r="2" spans="1:1024" ht="105.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>100</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
       <c r="AMG2" s="13"/>
       <c r="AMH2" s="13"/>
       <c r="AMI2" s="13"/>
@@ -2856,13 +2856,13 @@
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -2897,74 +2897,74 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:1024" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:1024" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3009,7 +3009,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="39" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="C13" s="39"/>
       <c r="D13" s="39"/>
@@ -3017,7 +3017,7 @@
       <c r="F13" s="39"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
     </row>
     <row r="14" spans="1:1024" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -3057,10 +3057,10 @@
       <c r="B16" s="39" t="s">
         <v>115</v>
       </c>
-      <c r="C16" s="52"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="52"/>
-      <c r="F16" s="53"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="41"/>
+      <c r="F16" s="42"/>
       <c r="G16" s="9" t="s">
         <v>114</v>
       </c>
@@ -3181,14 +3181,14 @@
         <v>38</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="12" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="H22" s="17"/>
     </row>
@@ -3197,7 +3197,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>262</v>
+        <v>313</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>28</v>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="F23" s="10"/>
       <c r="G23" s="12" t="s">
-        <v>263</v>
+        <v>314</v>
       </c>
       <c r="H23" s="17"/>
     </row>
@@ -3219,7 +3219,7 @@
         <v>27</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>28</v>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="F24" s="10"/>
       <c r="G24" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="H24" s="17"/>
     </row>
@@ -3262,13 +3262,13 @@
       <c r="A26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B26" s="41" t="s">
+      <c r="B26" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="41"/>
-      <c r="D26" s="41"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
       <c r="G26" s="1" t="s">
         <v>6</v>
       </c>
@@ -3281,7 +3281,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="39" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="C27" s="39"/>
       <c r="D27" s="39"/>
@@ -3327,7 +3327,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="39" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="C30" s="39"/>
       <c r="D30" s="39"/>
@@ -3335,7 +3335,7 @@
       <c r="F30" s="39"/>
       <c r="G30" s="9"/>
       <c r="H30" s="9" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="F36" s="10"/>
       <c r="G36" s="12" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="H36" s="17"/>
     </row>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>262</v>
+        <v>313</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>28</v>
@@ -3482,7 +3482,7 @@
       </c>
       <c r="F37" s="10"/>
       <c r="G37" s="12" t="s">
-        <v>265</v>
+        <v>315</v>
       </c>
       <c r="H37" s="17"/>
     </row>
@@ -3491,7 +3491,7 @@
         <v>27</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>28</v>
@@ -3504,7 +3504,7 @@
       </c>
       <c r="F38" s="10"/>
       <c r="G38" s="2" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="H38" s="17"/>
     </row>
@@ -3534,13 +3534,13 @@
       <c r="A40" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B40" s="41" t="s">
+      <c r="B40" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C40" s="41"/>
-      <c r="D40" s="41"/>
-      <c r="E40" s="41"/>
-      <c r="F40" s="41"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="40"/>
       <c r="G40" s="1" t="s">
         <v>6</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>3</v>
       </c>
       <c r="B41" s="39" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="C41" s="39"/>
       <c r="D41" s="39"/>
@@ -3569,10 +3569,10 @@
       <c r="B42" s="39" t="s">
         <v>146</v>
       </c>
-      <c r="C42" s="52"/>
-      <c r="D42" s="52"/>
-      <c r="E42" s="52"/>
-      <c r="F42" s="53"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="41"/>
+      <c r="E42" s="41"/>
+      <c r="F42" s="42"/>
       <c r="G42" s="9" t="s">
         <v>145</v>
       </c>
@@ -3665,7 +3665,7 @@
         <v>27</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>28</v>
@@ -3686,13 +3686,13 @@
       <c r="A48" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B48" s="41" t="s">
+      <c r="B48" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
+      <c r="C48" s="40"/>
+      <c r="D48" s="40"/>
+      <c r="E48" s="40"/>
+      <c r="F48" s="40"/>
       <c r="G48" s="1" t="s">
         <v>6</v>
       </c>
@@ -3707,10 +3707,10 @@
       <c r="B49" s="39" t="s">
         <v>148</v>
       </c>
-      <c r="C49" s="52"/>
-      <c r="D49" s="52"/>
-      <c r="E49" s="52"/>
-      <c r="F49" s="53"/>
+      <c r="C49" s="41"/>
+      <c r="D49" s="41"/>
+      <c r="E49" s="41"/>
+      <c r="F49" s="42"/>
       <c r="G49" s="9" t="s">
         <v>147</v>
       </c>
@@ -3721,7 +3721,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="39" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="C50" s="39"/>
       <c r="D50" s="39"/>
@@ -3734,13 +3734,13 @@
       <c r="A51" s="8">
         <v>4</v>
       </c>
-      <c r="B51" s="54" t="s">
+      <c r="B51" s="43" t="s">
         <v>69</v>
       </c>
-      <c r="C51" s="52"/>
-      <c r="D51" s="52"/>
-      <c r="E51" s="52"/>
-      <c r="F51" s="53"/>
+      <c r="C51" s="41"/>
+      <c r="D51" s="41"/>
+      <c r="E51" s="41"/>
+      <c r="F51" s="42"/>
       <c r="G51" s="9"/>
       <c r="H51" s="17"/>
     </row>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>28</v>
@@ -3896,12 +3896,33 @@
       </c>
       <c r="F58" s="10"/>
       <c r="G58" s="2" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="H58" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B50:F50"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="B49:F49"/>
@@ -3918,27 +3939,6 @@
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="B31:F31"/>
     <mergeCell ref="B40:F40"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B13:F13"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3967,40 +3967,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
       <c r="AMI1" s="13"/>
       <c r="AMJ1" s="13"/>
     </row>
     <row r="2" spans="1:1024" ht="104.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
       <c r="AMI2" s="13"/>
       <c r="AMJ2" s="13"/>
     </row>
@@ -4008,13 +4008,13 @@
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4049,14 +4049,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -4069,60 +4069,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:1024" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:1024" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -4151,7 +4151,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="39" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="C12" s="39"/>
       <c r="D12" s="39"/>
@@ -4337,7 +4337,7 @@
         <v>27</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>262</v>
+        <v>313</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>28</v>
@@ -4350,7 +4350,7 @@
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="12" t="s">
-        <v>268</v>
+        <v>316</v>
       </c>
       <c r="H22" s="17"/>
     </row>
@@ -4359,7 +4359,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>28</v>
@@ -4372,7 +4372,7 @@
       </c>
       <c r="F23" s="10"/>
       <c r="G23" s="2" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="H23" s="17"/>
     </row>
@@ -4380,13 +4380,13 @@
       <c r="A24" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B24" s="41" t="s">
+      <c r="B24" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
       <c r="G24" s="1" t="s">
         <v>6</v>
       </c>
@@ -4399,7 +4399,7 @@
         <v>2</v>
       </c>
       <c r="B25" s="39" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="C25" s="39"/>
       <c r="D25" s="39"/>
@@ -4413,7 +4413,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="39" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="C26" s="39"/>
       <c r="D26" s="39"/>
@@ -4443,7 +4443,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -4604,13 +4604,13 @@
       <c r="A36" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B36" s="41" t="s">
+      <c r="B36" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="41"/>
-      <c r="D36" s="41"/>
-      <c r="E36" s="41"/>
-      <c r="F36" s="41"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="40"/>
+      <c r="E36" s="40"/>
+      <c r="F36" s="40"/>
       <c r="G36" s="1" t="s">
         <v>6</v>
       </c>
@@ -4623,7 +4623,7 @@
         <v>3</v>
       </c>
       <c r="B37" s="39" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="C37" s="39"/>
       <c r="D37" s="39"/>
@@ -4636,13 +4636,13 @@
       <c r="A38" s="8">
         <v>3</v>
       </c>
-      <c r="B38" s="54" t="s">
+      <c r="B38" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="C38" s="52"/>
-      <c r="D38" s="52"/>
-      <c r="E38" s="52"/>
-      <c r="F38" s="53"/>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="41"/>
+      <c r="F38" s="42"/>
       <c r="G38" s="9" t="s">
         <v>152</v>
       </c>
@@ -4653,7 +4653,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="39" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C39" s="39"/>
       <c r="D39" s="39"/>
@@ -4812,27 +4812,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B38:F38"/>
@@ -4845,6 +4824,27 @@
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B37:F37"/>
     <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4873,50 +4873,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>112</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4951,14 +4951,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -4971,60 +4971,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="18" t="s">
         <v>6</v>
       </c>
@@ -5036,13 +5036,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="54" t="s">
+      <c r="B11" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="52"/>
-      <c r="D11" s="52"/>
-      <c r="E11" s="52"/>
-      <c r="F11" s="53"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="42"/>
       <c r="G11" s="19"/>
       <c r="H11" s="17" t="s">
         <v>22</v>
@@ -5052,13 +5052,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="54" t="s">
+      <c r="B12" s="43" t="s">
         <v>136</v>
       </c>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="53"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="42"/>
       <c r="G12" s="19"/>
       <c r="H12" s="17" t="s">
         <v>125</v>
@@ -5069,7 +5069,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="39" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="C13" s="39"/>
       <c r="D13" s="39"/>
@@ -5085,7 +5085,7 @@
         <v>1</v>
       </c>
       <c r="B14" s="39" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="C14" s="39"/>
       <c r="D14" s="39"/>
@@ -5093,7 +5093,7 @@
       <c r="F14" s="39"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -5257,14 +5257,14 @@
         <v>38</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F23" s="10"/>
       <c r="G23" s="12" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="H23" s="17"/>
     </row>
@@ -5273,7 +5273,7 @@
         <v>27</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>262</v>
+        <v>313</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="F24" s="10"/>
       <c r="G24" s="21" t="s">
-        <v>263</v>
+        <v>314</v>
       </c>
       <c r="H24" s="17"/>
     </row>
@@ -5295,7 +5295,7 @@
         <v>27</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>28</v>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="F25" s="10"/>
       <c r="G25" s="20" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="H25" s="17"/>
     </row>
@@ -5338,13 +5338,13 @@
       <c r="A27" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B27" s="41" t="s">
+      <c r="B27" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C27" s="41"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
       <c r="G27" s="18" t="s">
         <v>6</v>
       </c>
@@ -6373,7 +6373,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -8451,7 +8451,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="39" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="C31" s="39"/>
       <c r="D31" s="39"/>
@@ -9483,7 +9483,7 @@
         <v>2</v>
       </c>
       <c r="B32" s="39" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="C32" s="39"/>
       <c r="D32" s="39"/>
@@ -9491,7 +9491,7 @@
       <c r="F32" s="39"/>
       <c r="G32" s="9"/>
       <c r="H32" s="9" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
     </row>
     <row r="33" spans="1:1024" x14ac:dyDescent="0.2">
@@ -11640,14 +11640,14 @@
         <v>38</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="E38" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F38" s="10"/>
       <c r="G38" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H38" s="17"/>
     </row>
@@ -11656,7 +11656,7 @@
         <v>27</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>262</v>
+        <v>313</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>28</v>
@@ -11669,7 +11669,7 @@
       </c>
       <c r="F39" s="10"/>
       <c r="G39" s="21" t="s">
-        <v>270</v>
+        <v>317</v>
       </c>
       <c r="H39" s="17"/>
     </row>
@@ -11678,7 +11678,7 @@
         <v>27</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>28</v>
@@ -11691,7 +11691,7 @@
       </c>
       <c r="F40" s="10"/>
       <c r="G40" s="20" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="H40" s="17"/>
     </row>
@@ -11721,13 +11721,13 @@
       <c r="A42" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B42" s="41" t="s">
+      <c r="B42" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C42" s="41"/>
-      <c r="D42" s="41"/>
-      <c r="E42" s="41"/>
-      <c r="F42" s="41"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="40"/>
+      <c r="E42" s="40"/>
+      <c r="F42" s="40"/>
       <c r="G42" s="18" t="s">
         <v>6</v>
       </c>
@@ -12756,7 +12756,7 @@
         <v>3</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C43" s="39"/>
       <c r="D43" s="39"/>
@@ -15915,13 +15915,13 @@
       <c r="A49" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B49" s="41" t="s">
+      <c r="B49" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="41"/>
-      <c r="D49" s="41"/>
-      <c r="E49" s="41"/>
-      <c r="F49" s="41"/>
+      <c r="C49" s="40"/>
+      <c r="D49" s="40"/>
+      <c r="E49" s="40"/>
+      <c r="F49" s="40"/>
       <c r="G49" s="18" t="s">
         <v>6</v>
       </c>
@@ -17982,7 +17982,7 @@
         <v>4</v>
       </c>
       <c r="B51" s="39" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="C51" s="39"/>
       <c r="D51" s="39"/>
@@ -20107,29 +20107,6 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B50:F50"/>
     <mergeCell ref="B52:F52"/>
     <mergeCell ref="B17:F17"/>
@@ -20146,6 +20123,29 @@
     <mergeCell ref="B45:F45"/>
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B33:F33"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -20174,50 +20174,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="154.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>111</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -20252,14 +20252,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -20272,60 +20272,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -20353,13 +20353,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="54" t="s">
+      <c r="B12" s="43" t="s">
         <v>142</v>
       </c>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="53"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="42"/>
       <c r="G12" s="9"/>
       <c r="H12" s="17" t="s">
         <v>125</v>
@@ -20386,7 +20386,7 @@
         <v>1</v>
       </c>
       <c r="B14" s="39" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="C14" s="39"/>
       <c r="D14" s="39"/>
@@ -20394,7 +20394,7 @@
       <c r="F14" s="39"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -20434,10 +20434,10 @@
       <c r="B17" s="39" t="s">
         <v>135</v>
       </c>
-      <c r="C17" s="52"/>
-      <c r="D17" s="52"/>
-      <c r="E17" s="52"/>
-      <c r="F17" s="53"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="42"/>
       <c r="G17" s="9" t="s">
         <v>134</v>
       </c>
@@ -20565,7 +20565,7 @@
       </c>
       <c r="F23" s="10"/>
       <c r="G23" s="12" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="H23" s="17"/>
     </row>
@@ -20574,7 +20574,7 @@
         <v>27</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>262</v>
+        <v>313</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>28</v>
@@ -20587,7 +20587,7 @@
       </c>
       <c r="F24" s="10"/>
       <c r="G24" s="12" t="s">
-        <v>265</v>
+        <v>315</v>
       </c>
       <c r="H24" s="17"/>
     </row>
@@ -20596,7 +20596,7 @@
         <v>27</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>28</v>
@@ -20609,7 +20609,7 @@
       </c>
       <c r="F25" s="10"/>
       <c r="G25" s="2" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="H25" s="17"/>
     </row>
@@ -20639,13 +20639,13 @@
       <c r="A27" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B27" s="41" t="s">
+      <c r="B27" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C27" s="41"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
       <c r="G27" s="1" t="s">
         <v>6</v>
       </c>
@@ -20658,7 +20658,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -20688,7 +20688,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="39" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C30" s="39"/>
       <c r="D30" s="39"/>
@@ -20858,7 +20858,7 @@
         <v>42</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E38" s="10" t="s">
         <v>29</v>
@@ -20880,7 +20880,7 @@
         <v>42</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>29</v>
@@ -20895,13 +20895,13 @@
       <c r="A40" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B40" s="41" t="s">
+      <c r="B40" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C40" s="41"/>
-      <c r="D40" s="41"/>
-      <c r="E40" s="41"/>
-      <c r="F40" s="41"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="40"/>
       <c r="G40" s="1" t="s">
         <v>6</v>
       </c>
@@ -20914,7 +20914,7 @@
         <v>3</v>
       </c>
       <c r="B41" s="39" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C41" s="39"/>
       <c r="D41" s="39"/>
@@ -20962,7 +20962,7 @@
         <v>3</v>
       </c>
       <c r="B44" s="39" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="C44" s="39"/>
       <c r="D44" s="39"/>
@@ -21130,7 +21130,7 @@
         <v>42</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E52" s="10" t="s">
         <v>29</v>
@@ -21152,7 +21152,7 @@
         <v>42</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>29</v>
@@ -21165,28 +21165,6 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B42:F42"/>
     <mergeCell ref="B45:F45"/>
@@ -21200,6 +21178,28 @@
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -21228,50 +21228,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>258</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>110</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -21306,14 +21306,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -21326,60 +21326,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -21424,7 +21424,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="39" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="C13" s="39"/>
       <c r="D13" s="39"/>
@@ -21432,7 +21432,7 @@
       <c r="F13" s="39"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -21454,14 +21454,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>315</v>
-      </c>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="53"/>
+        <v>309</v>
+      </c>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="42"/>
       <c r="G15" s="9" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="H15" s="17"/>
     </row>
@@ -21580,14 +21580,14 @@
         <v>38</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F21" s="10"/>
       <c r="G21" s="12" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="H21" s="17"/>
     </row>
@@ -21596,7 +21596,7 @@
         <v>27</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>262</v>
+        <v>313</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>28</v>
@@ -21609,7 +21609,7 @@
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="12" t="s">
-        <v>263</v>
+        <v>314</v>
       </c>
       <c r="H22" s="17"/>
     </row>
@@ -21618,7 +21618,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>28</v>
@@ -21631,7 +21631,7 @@
       </c>
       <c r="F23" s="10"/>
       <c r="G23" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="H23" s="17"/>
     </row>
@@ -21661,13 +21661,13 @@
       <c r="A25" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B25" s="41" t="s">
+      <c r="B25" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C25" s="41"/>
-      <c r="D25" s="41"/>
-      <c r="E25" s="41"/>
-      <c r="F25" s="41"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
       <c r="G25" s="1" t="s">
         <v>6</v>
       </c>
@@ -21680,7 +21680,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="39" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C26" s="39"/>
       <c r="D26" s="39"/>
@@ -21710,7 +21710,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -21873,13 +21873,13 @@
       <c r="A36" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B36" s="41" t="s">
+      <c r="B36" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="41"/>
-      <c r="D36" s="41"/>
-      <c r="E36" s="41"/>
-      <c r="F36" s="41"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="40"/>
+      <c r="E36" s="40"/>
+      <c r="F36" s="40"/>
       <c r="G36" s="1" t="s">
         <v>6</v>
       </c>
@@ -21892,7 +21892,7 @@
         <v>3</v>
       </c>
       <c r="B37" s="39" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="C37" s="39"/>
       <c r="D37" s="39"/>
@@ -21922,7 +21922,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="39" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C39" s="39"/>
       <c r="D39" s="39"/>
@@ -22083,28 +22083,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="B13:F13"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B16:F16"/>
@@ -22115,6 +22093,28 @@
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B37:F37"/>
     <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -22143,50 +22143,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="160.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>109</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -22221,14 +22221,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -22241,60 +22241,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -22323,7 +22323,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="39" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="C12" s="39"/>
       <c r="D12" s="39"/>
@@ -22339,7 +22339,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="39" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="C13" s="39"/>
       <c r="D13" s="39"/>
@@ -22347,7 +22347,7 @@
       <c r="F13" s="39"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -22368,13 +22368,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="54" t="s">
+      <c r="B15" s="43" t="s">
         <v>143</v>
       </c>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="53"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="42"/>
       <c r="G15" s="9" t="s">
         <v>158</v>
       </c>
@@ -22482,7 +22482,7 @@
       </c>
       <c r="F20" s="10"/>
       <c r="G20" s="12" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="H20" s="17"/>
     </row>
@@ -22491,7 +22491,7 @@
         <v>27</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>262</v>
+        <v>313</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>28</v>
@@ -22504,7 +22504,7 @@
       </c>
       <c r="F21" s="10"/>
       <c r="G21" s="12" t="s">
-        <v>265</v>
+        <v>315</v>
       </c>
       <c r="H21" s="17"/>
     </row>
@@ -22513,7 +22513,7 @@
         <v>27</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>28</v>
@@ -22526,7 +22526,7 @@
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="2" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="H22" s="17"/>
     </row>
@@ -22556,13 +22556,13 @@
       <c r="A24" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B24" s="41" t="s">
+      <c r="B24" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
       <c r="G24" s="1" t="s">
         <v>6</v>
       </c>
@@ -22575,7 +22575,7 @@
         <v>2</v>
       </c>
       <c r="B25" s="39" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C25" s="39"/>
       <c r="D25" s="39"/>
@@ -22605,7 +22605,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="39" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="C27" s="39"/>
       <c r="D27" s="39"/>
@@ -22724,13 +22724,13 @@
       <c r="A33" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B33" s="41" t="s">
+      <c r="B33" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="40"/>
+      <c r="E33" s="40"/>
+      <c r="F33" s="40"/>
       <c r="G33" s="1" t="s">
         <v>6</v>
       </c>
@@ -22743,7 +22743,7 @@
         <v>3</v>
       </c>
       <c r="B34" s="39" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="C34" s="39"/>
       <c r="D34" s="39"/>
@@ -22773,7 +22773,7 @@
         <v>3</v>
       </c>
       <c r="B36" s="39" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="C36" s="39"/>
       <c r="D36" s="39"/>
@@ -22786,13 +22786,13 @@
       <c r="A37" s="8">
         <v>3</v>
       </c>
-      <c r="B37" s="54" t="s">
+      <c r="B37" s="43" t="s">
         <v>69</v>
       </c>
-      <c r="C37" s="52"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="52"/>
-      <c r="F37" s="53"/>
+      <c r="C37" s="41"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="41"/>
+      <c r="F37" s="42"/>
       <c r="G37" s="9" t="s">
         <v>119</v>
       </c>
@@ -22890,28 +22890,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B35:F35"/>
-    <mergeCell ref="B13:F13"/>
     <mergeCell ref="B37:F37"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B24:F24"/>
@@ -22922,6 +22900,28 @@
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B34:F34"/>
     <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -22950,50 +22950,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="129" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>105</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -23028,14 +23028,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -23048,60 +23048,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -23129,13 +23129,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="54" t="s">
+      <c r="B12" s="43" t="s">
         <v>144</v>
       </c>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="53"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="42"/>
       <c r="G12" s="9"/>
       <c r="H12" s="17" t="s">
         <v>125</v>
@@ -23162,7 +23162,7 @@
         <v>1</v>
       </c>
       <c r="B14" s="39" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="C14" s="39"/>
       <c r="D14" s="39"/>
@@ -23170,7 +23170,7 @@
       <c r="F14" s="39"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="41.85" customHeight="1" x14ac:dyDescent="0.2">
@@ -23192,14 +23192,14 @@
         <v>1</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="C16" s="39"/>
       <c r="D16" s="39"/>
       <c r="E16" s="39"/>
       <c r="F16" s="39"/>
       <c r="G16" s="9" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="H16" s="17"/>
     </row>
@@ -23318,14 +23318,14 @@
         <v>38</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="12" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="H22" s="17"/>
     </row>
@@ -23334,7 +23334,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>262</v>
+        <v>313</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>28</v>
@@ -23347,7 +23347,7 @@
       </c>
       <c r="F23" s="10"/>
       <c r="G23" s="12" t="s">
-        <v>263</v>
+        <v>314</v>
       </c>
       <c r="H23" s="17"/>
     </row>
@@ -23356,7 +23356,7 @@
         <v>27</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>28</v>
@@ -23369,7 +23369,7 @@
       </c>
       <c r="F24" s="10"/>
       <c r="G24" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="H24" s="17"/>
     </row>
@@ -23399,13 +23399,13 @@
       <c r="A26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B26" s="41" t="s">
+      <c r="B26" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="41"/>
-      <c r="D26" s="41"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
       <c r="G26" s="1" t="s">
         <v>6</v>
       </c>
@@ -23418,7 +23418,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="39" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="C27" s="39"/>
       <c r="D27" s="39"/>
@@ -23448,7 +23448,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="39" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="C29" s="39"/>
       <c r="D29" s="39"/>
@@ -23462,7 +23462,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="39" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="C30" s="39"/>
       <c r="D30" s="39"/>
@@ -23567,13 +23567,13 @@
       <c r="A35" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B35" s="41" t="s">
+      <c r="B35" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="41"/>
-      <c r="D35" s="41"/>
-      <c r="E35" s="41"/>
-      <c r="F35" s="41"/>
+      <c r="C35" s="40"/>
+      <c r="D35" s="40"/>
+      <c r="E35" s="40"/>
+      <c r="F35" s="40"/>
       <c r="G35" s="1" t="s">
         <v>6</v>
       </c>
@@ -23586,7 +23586,7 @@
         <v>3</v>
       </c>
       <c r="B36" s="39" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="C36" s="39"/>
       <c r="D36" s="39"/>
@@ -23616,7 +23616,7 @@
         <v>3</v>
       </c>
       <c r="B38" s="39" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="C38" s="39"/>
       <c r="D38" s="39"/>
@@ -23733,28 +23733,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B35:F35"/>
     <mergeCell ref="B37:F37"/>
     <mergeCell ref="B39:F39"/>
@@ -23766,6 +23744,28 @@
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="B36:F36"/>
     <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>